<commit_message>
[26 27] update transkrypcja_whishper.py
</commit_message>
<xml_diff>
--- a/day_23_20_09_2025/fix2.xlsx
+++ b/day_23_20_09_2025/fix2.xlsx
@@ -1,16 +1,114 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/radoslawjaniak/PycharmProjects/Bootcamp-10-05-2025/day_23_20_09_2025/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B332E8-9C2E-F644-A7C4-750DA87C4046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-34560" yWindow="-14180" windowWidth="27720" windowHeight="13580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="2">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+  <valueMetadata count="2">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
+<file path=xl/python.xml><?xml version="1.0" encoding="utf-8"?>
+<python xmlns="http://schemas.microsoft.com/office/spreadsheetml/2023/python">
+  <environmentDefinition id="{882DD1B0-6546-4DFA-8A08-902A380B44EA}">
+    <initialization>
+      <code xml:space="preserve">import numpy as np
+import pandas as pd
+import matplotlib.pyplot as plt
+import seaborn as sns
+import statsmodels as sm
+import excel
+import warnings
+warnings.simplefilter('ignore')
+excel.set_xl_scalar_conversion(excel.convert_to_scalar)
+excel.set_xl_array_conversion(excel.convert_to_dataframe)
+</code>
+    </initialization>
+  </environmentDefinition>
+  <pythonScripts>
+    <pythonScript>
+      <code>pd.DataFrame([1,2])</code>
+    </pythonScript>
+    <pythonScript>
+      <code>[1,2]</code>
+    </pythonScript>
+    <pythonScript>
+      <code>xl(%P2%)+xl(%P3%)[1,2]</code>
+    </pythonScript>
+  </pythonScripts>
+</python>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -67,8 +165,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,13 +229,192 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdarray.xml><?xml version="1.0" encoding="utf-8"?>
+<arrayData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="2">
+  <a r="3" c="2">
+    <v t="s"/>
+    <v>0</v>
+    <v>0</v>
+    <v>1</v>
+    <v>1</v>
+    <v>2</v>
+  </a>
+  <a r="2">
+    <v>1</v>
+    <v>2</v>
+  </a>
+</arrayData>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
+  <rv s="0">
+    <v>0</v>
+  </rv>
+  <rv s="1">
+    <v>DataFrame</v>
+    <v>1</v>
+    <v>0</v>
+  </rv>
+  <rv s="2">
+    <v>&lt;class 'pandas.core.frame.DataFrame'&gt;</v>
+    <v>DataFrame</v>
+    <v xml:space="preserve">   0
+0  1
+1  2</v>
+    <v>1</v>
+    <v>2</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+  </rv>
+  <rv s="1">
+    <v>list</v>
+    <v>4</v>
+    <v>3</v>
+  </rv>
+  <rv s="2">
+    <v>&lt;class 'list'&gt;</v>
+    <v>list</v>
+    <v>[1, 2]</v>
+    <v>4</v>
+    <v>2</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3">
+  <s t="_array">
+    <k n="array" t="a"/>
+  </s>
+  <s t="_entity">
+    <k n="_DisplayString" t="s"/>
+    <k n="_ViewInfo" t="spb"/>
+    <k n="arrayPreview" t="r"/>
+  </s>
+  <s t="_python">
+    <k n="Python_type" t="s"/>
+    <k n="Python_typeName" t="s"/>
+    <k n="Python_str" t="s"/>
+    <k n="preview" t="r"/>
+    <k n="_Provider" t="spb"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
+<supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
+  <spbData count="5">
+    <spb s="0">
+      <v>2</v>
+      <v>1</v>
+      <v>DataFrame</v>
+      <v>arrayPreview</v>
+      <v>1</v>
+    </spb>
+    <spb s="1">
+      <v>0</v>
+    </spb>
+    <spb s="2">
+      <v>https://www.anaconda.com/excel</v>
+      <v>https://res.cdn.office.net/officepysvc/prod-service/anacondalogo.png</v>
+      <v>Python provided by Anaconda</v>
+    </spb>
+    <spb s="3">
+      <v>2</v>
+      <v>1</v>
+      <v>list</v>
+      <v>arrayPreview</v>
+    </spb>
+    <spb s="1">
+      <v>3</v>
+    </spb>
+  </spbData>
+</supportingPropertyBags>
+</file>
+
+<file path=xl/richData/rdsupportingpropertybagstructure.xml><?xml version="1.0" encoding="utf-8"?>
+<spbStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="4">
+  <s>
+    <k n="drw" t="i"/>
+    <k n="dcol" t="i"/>
+    <k n="name" t="s"/>
+    <k n="array" t="s"/>
+    <k n="headers" t="b"/>
+  </s>
+  <s>
+    <k n="ArrayCardInfo" t="spb"/>
+  </s>
+  <s>
+    <k n="link" t="s"/>
+    <k n="logo" t="s"/>
+    <k n="name" t="s"/>
+  </s>
+  <s>
+    <k n="drw" t="i"/>
+    <k n="dcol" t="i"/>
+    <k n="name" t="s"/>
+    <k n="array" t="s"/>
+  </s>
+</spbStructures>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -175,7 +452,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -209,6 +486,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -243,9 +521,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -418,11 +697,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1">
         <v>0</v>
       </c>
@@ -433,7 +712,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -444,7 +723,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -455,7 +734,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -466,7 +745,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -477,7 +756,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -488,7 +767,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -499,7 +778,7 @@
         <v>22000</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -510,7 +789,7 @@
         <v>19500</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -521,7 +800,7 @@
         <v>10500</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -532,7 +811,7 @@
         <v>17500</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -543,7 +822,7 @@
         <v>16000</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -554,7 +833,7 @@
         <v>14000</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -563,6 +842,55 @@
       </c>
       <c r="C15">
         <v>13000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C83609F6-5521-6540-A9F9-DCF716633114}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <f>PY1+2</f>
+        <v>2</v>
+      </c>
+      <c r="B1" t="e" cm="1" vm="1">
+        <f t="array" ref="B1">_xlfn._xlws.PY(0,1)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C1" t="e" cm="1" vm="1">
+        <f t="array" ref="C1">_xlfn._xlws.PY(0,1)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B3" t="e" cm="1" vm="2">
+        <f t="array" ref="B3">_xlfn._xlws.PY(1,1)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C3" t="e" cm="1" vm="2">
+        <f t="array" ref="C3">_xlfn._xlws.PY(1,1)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C4" t="e" cm="1" vm="2">
+        <f t="array" ref="C4">_xlfn._xlws.PY(1,1)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B7" cm="1">
+        <f t="array" aca="1" ref="B7" ca="1">_xlfn._xlws.PY(2,1,B7,B9)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>